<commit_message>
fix(hardware): 移除 V4.11 MARK 并同步贴片助手
</commit_message>
<xml_diff>
--- a/hardware/expansion-board-v4/CHECKLIST-V4.11.xlsx
+++ b/hardware/expansion-board-v4/CHECKLIST-V4.11.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V4.11 核对清单" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="V4.11 核对清单" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'V4.11 核对清单'!$1:$1</definedName>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G256"/>
+  <dimension ref="A1:G252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -7492,106 +7492,30 @@
       <c r="A252" s="2" t="inlineStr"/>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>FID1</t>
+          <t>RT1</t>
         </is>
       </c>
       <c r="C252" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D252" s="4" t="inlineStr"/>
+          <t>NCP18XH103F03RB 10k NTC</t>
+        </is>
+      </c>
+      <c r="D252" s="4" t="inlineStr">
+        <is>
+          <t>R_0603_1608Metric</t>
+        </is>
+      </c>
       <c r="E252" s="2" t="inlineStr">
         <is>
-          <t>59.2, 56.0</t>
+          <t>54.8, 100.9</t>
         </is>
       </c>
       <c r="F252" s="4" t="inlineStr">
         <is>
-          <t>? ?</t>
+          <t>A 电源</t>
         </is>
       </c>
       <c r="G252" s="5" t="inlineStr"/>
-    </row>
-    <row r="253" ht="19" customHeight="1">
-      <c r="A253" s="2" t="inlineStr"/>
-      <c r="B253" s="3" t="inlineStr">
-        <is>
-          <t>FID2</t>
-        </is>
-      </c>
-      <c r="C253" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D253" s="4" t="inlineStr"/>
-      <c r="E253" s="2" t="inlineStr">
-        <is>
-          <t>140.8, 56.0</t>
-        </is>
-      </c>
-      <c r="F253" s="4" t="inlineStr">
-        <is>
-          <t>? ?</t>
-        </is>
-      </c>
-      <c r="G253" s="5" t="inlineStr"/>
-    </row>
-    <row r="254" ht="19" customHeight="1">
-      <c r="A254" s="2" t="inlineStr"/>
-      <c r="B254" s="3" t="inlineStr">
-        <is>
-          <t>FID3</t>
-        </is>
-      </c>
-      <c r="C254" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D254" s="4" t="inlineStr"/>
-      <c r="E254" s="2" t="inlineStr">
-        <is>
-          <t>62.2, 106.5</t>
-        </is>
-      </c>
-      <c r="F254" s="4" t="inlineStr">
-        <is>
-          <t>? ?</t>
-        </is>
-      </c>
-      <c r="G254" s="5" t="inlineStr"/>
-    </row>
-    <row r="255" ht="19" customHeight="1"/>
-    <row r="256" ht="19" customHeight="1">
-      <c r="A256" s="2" t="inlineStr"/>
-      <c r="B256" s="3" t="inlineStr">
-        <is>
-          <t>RT1</t>
-        </is>
-      </c>
-      <c r="C256" s="4" t="inlineStr">
-        <is>
-          <t>NCP18XH103F03RB 10k NTC</t>
-        </is>
-      </c>
-      <c r="D256" s="4" t="inlineStr">
-        <is>
-          <t>R_0603_1608Metric</t>
-        </is>
-      </c>
-      <c r="E256" s="2" t="inlineStr">
-        <is>
-          <t>54.8, 100.9</t>
-        </is>
-      </c>
-      <c r="F256" s="4" t="inlineStr">
-        <is>
-          <t>A 电源</t>
-        </is>
-      </c>
-      <c r="G256" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <printOptions gridLines="0"/>

</xml_diff>